<commit_message>
Add replay CLI workflow routing and tests
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10302"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C936EB6-0E68-F747-B10B-C14DC3BDBB80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E78204F-5AC4-3141-B347-7B57C4BBBCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -1368,15 +1368,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1391,6 +1382,15 @@
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1931,53 +1931,53 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:34" ht="58.5" customHeight="1">
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="94"/>
-      <c r="M2" s="94"/>
-      <c r="N2" s="94"/>
-      <c r="O2" s="94"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="91"/>
+      <c r="K2" s="91"/>
+      <c r="L2" s="91"/>
+      <c r="M2" s="91"/>
+      <c r="N2" s="91"/>
+      <c r="O2" s="91"/>
       <c r="R2" s="36"/>
       <c r="U2" s="36"/>
       <c r="X2" s="36"/>
     </row>
     <row r="3" spans="1:34" ht="24.75" customHeight="1">
-      <c r="A3" s="93" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="93"/>
-      <c r="C3" s="93"/>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93"/>
+      <c r="A3" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
+      <c r="M3" s="90"/>
+      <c r="N3" s="90"/>
+      <c r="O3" s="90"/>
     </row>
     <row r="4" spans="1:34" ht="15" customHeight="1">
-      <c r="A4" s="93"/>
-      <c r="B4" s="93"/>
-      <c r="C4" s="93"/>
-      <c r="D4" s="93"/>
-      <c r="E4" s="93"/>
-      <c r="F4" s="93"/>
-      <c r="G4" s="93"/>
-      <c r="H4" s="93"/>
-      <c r="I4" s="93"/>
-      <c r="J4" s="93"/>
-      <c r="K4" s="93"/>
-      <c r="L4" s="93"/>
-      <c r="M4" s="93"/>
-      <c r="N4" s="93"/>
-      <c r="O4" s="93"/>
+      <c r="A4" s="90"/>
+      <c r="B4" s="90"/>
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="90"/>
+      <c r="L4" s="90"/>
+      <c r="M4" s="90"/>
+      <c r="N4" s="90"/>
+      <c r="O4" s="90"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="B6" s="77" t="s">
@@ -1989,15 +1989,15 @@
       <c r="B7" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="90" t="s">
+      <c r="E7" s="87" t="s">
         <v>48</v>
       </c>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="91"/>
-      <c r="K7" s="92"/>
+      <c r="F7" s="88"/>
+      <c r="G7" s="88"/>
+      <c r="H7" s="88"/>
+      <c r="I7" s="88"/>
+      <c r="J7" s="88"/>
+      <c r="K7" s="89"/>
       <c r="L7" s="79"/>
       <c r="AH7" s="2"/>
     </row>
@@ -2005,15 +2005,15 @@
       <c r="B8" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="90" t="s">
+      <c r="E8" s="87" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="91"/>
-      <c r="G8" s="91"/>
-      <c r="H8" s="91"/>
-      <c r="I8" s="91"/>
-      <c r="J8" s="91"/>
-      <c r="K8" s="92"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="88"/>
+      <c r="K8" s="89"/>
       <c r="L8" s="79"/>
       <c r="AH8" s="2"/>
     </row>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="E12" s="70">
         <f>March!AH14</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F12" s="70">
         <f>April!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>159</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="E29" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>159</v>
+        <v>199</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -3198,34 +3198,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -3236,32 +3236,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -4326,34 +4326,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -4364,32 +4364,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -5473,34 +5473,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -5511,32 +5511,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -6596,34 +6596,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -6634,32 +6634,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -7750,34 +7750,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:37" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:37" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -7788,32 +7788,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:37" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:37" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -8911,34 +8911,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:31" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:31" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -8949,32 +8949,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:31" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:31" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -10031,34 +10031,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -10069,32 +10069,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -10238,15 +10238,31 @@
         <f>January!B14</f>
         <v>AI-Driven Agentic Orchestration Software (AOC-WebAPI)</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
+      <c r="C14" s="16">
+        <v>6</v>
+      </c>
+      <c r="D14" s="17">
+        <v>5</v>
+      </c>
+      <c r="E14" s="17">
+        <v>6</v>
+      </c>
+      <c r="F14" s="17">
+        <v>5</v>
+      </c>
       <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="17"/>
+      <c r="H14" s="17">
+        <v>4</v>
+      </c>
+      <c r="I14" s="18">
+        <v>4</v>
+      </c>
+      <c r="J14" s="16">
+        <v>2</v>
+      </c>
+      <c r="K14" s="17">
+        <v>8</v>
+      </c>
       <c r="L14" s="17"/>
       <c r="M14" s="17"/>
       <c r="N14" s="17"/>
@@ -10271,7 +10287,7 @@
       <c r="AG14" s="20"/>
       <c r="AH14" s="21">
         <f t="shared" ref="AH14:AH30" si="0">SUM(C14:AG14)</f>
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -11177,34 +11193,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -11215,32 +11231,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -12300,34 +12316,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -12338,32 +12354,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87" t="s">
+      <c r="C9" s="92" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -13447,34 +13463,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -13485,32 +13501,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -14569,34 +14585,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -14607,32 +14623,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -15719,34 +15735,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -15757,32 +15773,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -16829,14 +16845,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17075,23 +17089,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -17116,9 +17127,14 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Add HMAC-chained event log integrity and replay verification
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DA067B0-689E-E342-82F7-C58FBC4B4BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201D10F7-F416-4D48-9318-299180749CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="E12" s="70">
         <f>March!AH14</f>
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="F12" s="70">
         <f>April!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>231</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="E29" s="5">
         <f t="shared" si="1"/>
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="F29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>231</v>
+        <v>257</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -10285,13 +10285,25 @@
         <v>4</v>
       </c>
       <c r="S14" s="17"/>
-      <c r="T14" s="17"/>
-      <c r="U14" s="17"/>
-      <c r="V14" s="17"/>
+      <c r="T14" s="17">
+        <v>4</v>
+      </c>
+      <c r="U14" s="17">
+        <v>6</v>
+      </c>
+      <c r="V14" s="17">
+        <v>4</v>
+      </c>
       <c r="W14" s="18"/>
-      <c r="X14" s="16"/>
-      <c r="Y14" s="17"/>
-      <c r="Z14" s="17"/>
+      <c r="X14" s="16">
+        <v>4</v>
+      </c>
+      <c r="Y14" s="17">
+        <v>2</v>
+      </c>
+      <c r="Z14" s="17">
+        <v>6</v>
+      </c>
       <c r="AA14" s="17"/>
       <c r="AB14" s="17"/>
       <c r="AC14" s="17"/>
@@ -10301,7 +10313,7 @@
       <c r="AG14" s="20"/>
       <c r="AH14" s="21">
         <f t="shared" ref="AH14:AH30" si="0">SUM(C14:AG14)</f>
-        <v>72</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -16859,26 +16871,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17113,10 +17105,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -17135,20 +17158,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Complete March replay hardening with signed manifests and golden evaluation harness
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10404"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201D10F7-F416-4D48-9318-299180749CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B22FCD3-974F-CF46-AD79-9872EA8E2B79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="E12" s="70">
         <f>March!AH14</f>
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="F12" s="70">
         <f>April!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>257</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="E29" s="5">
         <f t="shared" si="1"/>
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="F29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>257</v>
+        <v>279</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -10305,15 +10305,25 @@
         <v>6</v>
       </c>
       <c r="AA14" s="17"/>
-      <c r="AB14" s="17"/>
-      <c r="AC14" s="17"/>
-      <c r="AD14" s="18"/>
-      <c r="AE14" s="16"/>
-      <c r="AF14" s="19"/>
+      <c r="AB14" s="17">
+        <v>8</v>
+      </c>
+      <c r="AC14" s="17">
+        <v>4</v>
+      </c>
+      <c r="AD14" s="18">
+        <v>2</v>
+      </c>
+      <c r="AE14" s="16">
+        <v>4</v>
+      </c>
+      <c r="AF14" s="19">
+        <v>4</v>
+      </c>
       <c r="AG14" s="20"/>
       <c r="AH14" s="21">
         <f t="shared" ref="AH14:AH30" si="0">SUM(C14:AG14)</f>
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -16871,6 +16881,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17105,27 +17135,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17144,27 +17175,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Integrate router decisions into replay manifests
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10412"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{017A17AA-B570-F243-95AB-228BDC5FD9FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB7E7CD-67B0-2247-8BFC-A446B7173B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="F12" s="70">
         <f>April!AG14</f>
-        <v>28</v>
+        <v>83</v>
       </c>
       <c r="G12" s="70">
         <f>May!AH14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>307</v>
+        <v>362</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="F29" s="5">
         <f t="shared" si="1"/>
-        <v>28</v>
+        <v>83</v>
       </c>
       <c r="G29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>307</v>
+        <v>362</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -11453,19 +11453,41 @@
         <v>8</v>
       </c>
       <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
-      <c r="M14" s="18"/>
+      <c r="L14" s="17">
+        <v>6</v>
+      </c>
+      <c r="M14" s="18">
+        <v>6</v>
+      </c>
       <c r="N14" s="16"/>
-      <c r="O14" s="17"/>
-      <c r="P14" s="17"/>
-      <c r="Q14" s="17"/>
+      <c r="O14" s="17">
+        <v>5</v>
+      </c>
+      <c r="P14" s="17">
+        <v>6</v>
+      </c>
+      <c r="Q14" s="17">
+        <v>5</v>
+      </c>
       <c r="R14" s="17"/>
-      <c r="S14" s="17"/>
-      <c r="T14" s="18"/>
-      <c r="U14" s="16"/>
-      <c r="V14" s="17"/>
-      <c r="W14" s="17"/>
-      <c r="X14" s="17"/>
+      <c r="S14" s="17">
+        <v>7</v>
+      </c>
+      <c r="T14" s="18">
+        <v>5</v>
+      </c>
+      <c r="U14" s="16">
+        <v>3</v>
+      </c>
+      <c r="V14" s="17">
+        <v>2</v>
+      </c>
+      <c r="W14" s="17">
+        <v>4</v>
+      </c>
+      <c r="X14" s="17">
+        <v>6</v>
+      </c>
       <c r="Y14" s="17"/>
       <c r="Z14" s="17"/>
       <c r="AA14" s="18"/>
@@ -11476,7 +11498,7 @@
       <c r="AF14" s="20"/>
       <c r="AG14" s="43">
         <f t="shared" ref="AG14:AG30" si="0">SUM(C14:AF14)</f>
-        <v>28</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:33" ht="15" customHeight="1">
@@ -16891,15 +16913,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
@@ -16908,6 +16921,15 @@
     <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17146,14 +17168,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -17162,6 +17176,14 @@
     <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
     <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
     <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
refactor: extract shared core, document April planner spike, and prep router benchmarks
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10419"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB7E7CD-67B0-2247-8BFC-A446B7173B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B226D81-1176-4C4A-866B-B069D5F64AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="17620" tabRatio="666" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2079,11 +2079,11 @@
       </c>
       <c r="F12" s="70">
         <f>April!AG14</f>
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="G12" s="70">
         <f>May!AH14</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H12" s="70">
         <f>June!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>362</v>
+        <v>389</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3064,11 +3064,11 @@
       </c>
       <c r="F29" s="5">
         <f t="shared" si="1"/>
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="G29" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>362</v>
+        <v>389</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -11488,17 +11488,29 @@
       <c r="X14" s="17">
         <v>6</v>
       </c>
-      <c r="Y14" s="17"/>
-      <c r="Z14" s="17"/>
-      <c r="AA14" s="18"/>
+      <c r="Y14" s="17">
+        <v>2</v>
+      </c>
+      <c r="Z14" s="17">
+        <v>5</v>
+      </c>
+      <c r="AA14" s="18">
+        <v>4</v>
+      </c>
       <c r="AB14" s="16"/>
       <c r="AC14" s="17"/>
-      <c r="AD14" s="17"/>
-      <c r="AE14" s="17"/>
-      <c r="AF14" s="20"/>
+      <c r="AD14" s="17">
+        <v>3</v>
+      </c>
+      <c r="AE14" s="17">
+        <v>3</v>
+      </c>
+      <c r="AF14" s="20">
+        <v>4</v>
+      </c>
       <c r="AG14" s="43">
         <f t="shared" ref="AG14:AG30" si="0">SUM(C14:AF14)</f>
-        <v>83</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:33" ht="15" customHeight="1">
@@ -12593,8 +12605,12 @@
         <v>AI-Driven Agentic Orchestration Software (AOC-WebAPI)</v>
       </c>
       <c r="C14" s="41"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="16"/>
+      <c r="D14" s="18">
+        <v>4</v>
+      </c>
+      <c r="E14" s="16">
+        <v>2</v>
+      </c>
       <c r="F14" s="17"/>
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
@@ -12625,7 +12641,7 @@
       <c r="AG14" s="54"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -16913,26 +16929,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17167,28 +17163,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17207,6 +17202,27 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Add router benchmark baseline for May metrics work
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10503"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B226D81-1176-4C4A-866B-B069D5F64AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE8E8BF-6EAA-654B-96BF-6AD1F3EDFA4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="17620" tabRatio="666" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -1368,15 +1368,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1391,6 +1382,15 @@
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1931,53 +1931,53 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:34" ht="58.5" customHeight="1">
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="94"/>
-      <c r="M2" s="94"/>
-      <c r="N2" s="94"/>
-      <c r="O2" s="94"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="91"/>
+      <c r="K2" s="91"/>
+      <c r="L2" s="91"/>
+      <c r="M2" s="91"/>
+      <c r="N2" s="91"/>
+      <c r="O2" s="91"/>
       <c r="R2" s="36"/>
       <c r="U2" s="36"/>
       <c r="X2" s="36"/>
     </row>
     <row r="3" spans="1:34" ht="24.75" customHeight="1">
-      <c r="A3" s="93" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="93"/>
-      <c r="C3" s="93"/>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93"/>
+      <c r="A3" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
+      <c r="M3" s="90"/>
+      <c r="N3" s="90"/>
+      <c r="O3" s="90"/>
     </row>
     <row r="4" spans="1:34" ht="15" customHeight="1">
-      <c r="A4" s="93"/>
-      <c r="B4" s="93"/>
-      <c r="C4" s="93"/>
-      <c r="D4" s="93"/>
-      <c r="E4" s="93"/>
-      <c r="F4" s="93"/>
-      <c r="G4" s="93"/>
-      <c r="H4" s="93"/>
-      <c r="I4" s="93"/>
-      <c r="J4" s="93"/>
-      <c r="K4" s="93"/>
-      <c r="L4" s="93"/>
-      <c r="M4" s="93"/>
-      <c r="N4" s="93"/>
-      <c r="O4" s="93"/>
+      <c r="A4" s="90"/>
+      <c r="B4" s="90"/>
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="90"/>
+      <c r="L4" s="90"/>
+      <c r="M4" s="90"/>
+      <c r="N4" s="90"/>
+      <c r="O4" s="90"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="B6" s="77" t="s">
@@ -1989,15 +1989,15 @@
       <c r="B7" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="90" t="s">
+      <c r="E7" s="87" t="s">
         <v>48</v>
       </c>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="91"/>
-      <c r="K7" s="92"/>
+      <c r="F7" s="88"/>
+      <c r="G7" s="88"/>
+      <c r="H7" s="88"/>
+      <c r="I7" s="88"/>
+      <c r="J7" s="88"/>
+      <c r="K7" s="89"/>
       <c r="L7" s="79"/>
       <c r="AH7" s="2"/>
     </row>
@@ -2005,15 +2005,15 @@
       <c r="B8" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="90" t="s">
+      <c r="E8" s="87" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="91"/>
-      <c r="G8" s="91"/>
-      <c r="H8" s="91"/>
-      <c r="I8" s="91"/>
-      <c r="J8" s="91"/>
-      <c r="K8" s="92"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="88"/>
+      <c r="K8" s="89"/>
       <c r="L8" s="79"/>
       <c r="AH8" s="2"/>
     </row>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="G12" s="70">
         <f>May!AH14</f>
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="H12" s="70">
         <f>June!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>389</v>
+        <v>415</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="G29" s="5">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="H29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>389</v>
+        <v>415</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -3198,34 +3198,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -3236,32 +3236,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -4326,34 +4326,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -4364,32 +4364,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -5473,34 +5473,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -5511,32 +5511,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -6596,34 +6596,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -6634,32 +6634,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -7750,34 +7750,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:37" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:37" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -7788,32 +7788,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:37" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:37" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -8911,34 +8911,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:31" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:31" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -8949,32 +8949,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:31" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:31" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -10031,34 +10031,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -10069,32 +10069,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -11229,34 +11229,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -11267,32 +11267,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -12396,34 +12396,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -12434,32 +12434,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87" t="s">
+      <c r="C9" s="92" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -12611,14 +12611,30 @@
       <c r="E14" s="16">
         <v>2</v>
       </c>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="17"/>
+      <c r="F14" s="17">
+        <v>6</v>
+      </c>
+      <c r="G14" s="17">
+        <v>4</v>
+      </c>
+      <c r="H14" s="17">
+        <v>4</v>
+      </c>
+      <c r="I14" s="17">
+        <v>2</v>
+      </c>
+      <c r="J14" s="17">
+        <v>4</v>
+      </c>
+      <c r="K14" s="18">
+        <v>3</v>
+      </c>
+      <c r="L14" s="16">
+        <v>1</v>
+      </c>
+      <c r="M14" s="17">
+        <v>2</v>
+      </c>
       <c r="N14" s="17"/>
       <c r="O14" s="17"/>
       <c r="P14" s="42"/>
@@ -12641,7 +12657,7 @@
       <c r="AG14" s="54"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>6</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -13547,34 +13563,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -13585,32 +13601,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -14669,34 +14685,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -14707,32 +14723,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -15819,34 +15835,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -15857,32 +15873,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -16929,6 +16945,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17163,27 +17199,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17202,27 +17239,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Add router metrics store foundation
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE8E8BF-6EAA-654B-96BF-6AD1F3EDFA4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7216C93-69D1-3C4D-B747-ABEC0763985D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -1368,6 +1368,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1382,15 +1391,6 @@
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1931,53 +1931,53 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:34" ht="58.5" customHeight="1">
-      <c r="H2" s="91"/>
-      <c r="I2" s="91"/>
-      <c r="J2" s="91"/>
-      <c r="K2" s="91"/>
-      <c r="L2" s="91"/>
-      <c r="M2" s="91"/>
-      <c r="N2" s="91"/>
-      <c r="O2" s="91"/>
+      <c r="H2" s="94"/>
+      <c r="I2" s="94"/>
+      <c r="J2" s="94"/>
+      <c r="K2" s="94"/>
+      <c r="L2" s="94"/>
+      <c r="M2" s="94"/>
+      <c r="N2" s="94"/>
+      <c r="O2" s="94"/>
       <c r="R2" s="36"/>
       <c r="U2" s="36"/>
       <c r="X2" s="36"/>
     </row>
     <row r="3" spans="1:34" ht="24.75" customHeight="1">
-      <c r="A3" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="90"/>
-      <c r="K3" s="90"/>
-      <c r="L3" s="90"/>
-      <c r="M3" s="90"/>
-      <c r="N3" s="90"/>
-      <c r="O3" s="90"/>
+      <c r="A3" s="93" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="93"/>
+      <c r="C3" s="93"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="93"/>
+      <c r="J3" s="93"/>
+      <c r="K3" s="93"/>
+      <c r="L3" s="93"/>
+      <c r="M3" s="93"/>
+      <c r="N3" s="93"/>
+      <c r="O3" s="93"/>
     </row>
     <row r="4" spans="1:34" ht="15" customHeight="1">
-      <c r="A4" s="90"/>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="90"/>
-      <c r="I4" s="90"/>
-      <c r="J4" s="90"/>
-      <c r="K4" s="90"/>
-      <c r="L4" s="90"/>
-      <c r="M4" s="90"/>
-      <c r="N4" s="90"/>
-      <c r="O4" s="90"/>
+      <c r="A4" s="93"/>
+      <c r="B4" s="93"/>
+      <c r="C4" s="93"/>
+      <c r="D4" s="93"/>
+      <c r="E4" s="93"/>
+      <c r="F4" s="93"/>
+      <c r="G4" s="93"/>
+      <c r="H4" s="93"/>
+      <c r="I4" s="93"/>
+      <c r="J4" s="93"/>
+      <c r="K4" s="93"/>
+      <c r="L4" s="93"/>
+      <c r="M4" s="93"/>
+      <c r="N4" s="93"/>
+      <c r="O4" s="93"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="B6" s="77" t="s">
@@ -1989,15 +1989,15 @@
       <c r="B7" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="87" t="s">
+      <c r="E7" s="90" t="s">
         <v>48</v>
       </c>
-      <c r="F7" s="88"/>
-      <c r="G7" s="88"/>
-      <c r="H7" s="88"/>
-      <c r="I7" s="88"/>
-      <c r="J7" s="88"/>
-      <c r="K7" s="89"/>
+      <c r="F7" s="91"/>
+      <c r="G7" s="91"/>
+      <c r="H7" s="91"/>
+      <c r="I7" s="91"/>
+      <c r="J7" s="91"/>
+      <c r="K7" s="92"/>
       <c r="L7" s="79"/>
       <c r="AH7" s="2"/>
     </row>
@@ -2005,15 +2005,15 @@
       <c r="B8" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="87" t="s">
+      <c r="E8" s="90" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="88"/>
-      <c r="K8" s="89"/>
+      <c r="F8" s="91"/>
+      <c r="G8" s="91"/>
+      <c r="H8" s="91"/>
+      <c r="I8" s="91"/>
+      <c r="J8" s="91"/>
+      <c r="K8" s="92"/>
       <c r="L8" s="79"/>
       <c r="AH8" s="2"/>
     </row>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="G12" s="70">
         <f>May!AH14</f>
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="H12" s="70">
         <f>June!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>415</v>
+        <v>449</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="G29" s="5">
         <f t="shared" si="1"/>
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="H29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>415</v>
+        <v>449</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -3198,34 +3198,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -3236,32 +3236,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -4326,34 +4326,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -4364,32 +4364,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -5473,34 +5473,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -5511,32 +5511,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -6596,34 +6596,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -6634,32 +6634,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -7750,34 +7750,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:37" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:37" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -7788,32 +7788,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:37" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:37" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -8911,34 +8911,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:31" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:31" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -8949,32 +8949,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:31" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:31" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -10031,34 +10031,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -10069,32 +10069,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -11229,34 +11229,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -11267,32 +11267,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -12396,34 +12396,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -12434,32 +12434,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92" t="s">
+      <c r="C9" s="87" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -12635,14 +12635,28 @@
       <c r="M14" s="17">
         <v>2</v>
       </c>
-      <c r="N14" s="17"/>
-      <c r="O14" s="17"/>
+      <c r="N14" s="17">
+        <v>5</v>
+      </c>
+      <c r="O14" s="17">
+        <v>5</v>
+      </c>
       <c r="P14" s="42"/>
-      <c r="Q14" s="17"/>
-      <c r="R14" s="18"/>
-      <c r="S14" s="16"/>
-      <c r="T14" s="17"/>
-      <c r="U14" s="17"/>
+      <c r="Q14" s="17">
+        <v>7</v>
+      </c>
+      <c r="R14" s="18">
+        <v>3</v>
+      </c>
+      <c r="S14" s="16">
+        <v>4</v>
+      </c>
+      <c r="T14" s="17">
+        <v>6</v>
+      </c>
+      <c r="U14" s="17">
+        <v>4</v>
+      </c>
       <c r="V14" s="17"/>
       <c r="W14" s="17"/>
       <c r="X14" s="17"/>
@@ -12657,7 +12671,7 @@
       <c r="AG14" s="54"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>32</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -13563,34 +13577,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -13601,32 +13615,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -14685,34 +14699,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -14723,32 +14737,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -15835,34 +15849,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -15873,32 +15887,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -16945,26 +16959,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17199,28 +17193,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17239,6 +17232,27 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Complete May router metrics weighting
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10510"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7216C93-69D1-3C4D-B747-ABEC0763985D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C1391F-2F90-A044-A0CD-C9064BE099E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="G12" s="70">
         <f>May!AH14</f>
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="H12" s="70">
         <f>June!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>449</v>
+        <v>485</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="G29" s="5">
         <f t="shared" si="1"/>
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="H29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>449</v>
+        <v>485</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -12657,21 +12657,37 @@
       <c r="U14" s="17">
         <v>4</v>
       </c>
-      <c r="V14" s="17"/>
+      <c r="V14" s="17">
+        <v>6</v>
+      </c>
       <c r="W14" s="17"/>
-      <c r="X14" s="17"/>
-      <c r="Y14" s="18"/>
-      <c r="Z14" s="16"/>
+      <c r="X14" s="17">
+        <v>4</v>
+      </c>
+      <c r="Y14" s="18">
+        <v>6</v>
+      </c>
+      <c r="Z14" s="16">
+        <v>2</v>
+      </c>
       <c r="AA14" s="42"/>
-      <c r="AB14" s="17"/>
-      <c r="AC14" s="17"/>
-      <c r="AD14" s="17"/>
-      <c r="AE14" s="17"/>
+      <c r="AB14" s="17">
+        <v>5</v>
+      </c>
+      <c r="AC14" s="17">
+        <v>4</v>
+      </c>
+      <c r="AD14" s="17">
+        <v>5</v>
+      </c>
+      <c r="AE14" s="17">
+        <v>4</v>
+      </c>
       <c r="AF14" s="18"/>
       <c r="AG14" s="54"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>66</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -16959,6 +16975,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17193,17 +17220,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -17214,6 +17230,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17232,19 +17261,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Add June tool execution protocol with replay capture
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C1391F-2F90-A044-A0CD-C9064BE099E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{521992A5-7392-C54B-912C-07EBCFC6EF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2083,11 +2083,11 @@
       </c>
       <c r="G12" s="70">
         <f>May!AH14</f>
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H12" s="70">
         <f>June!AG14</f>
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="I12" s="70">
         <f>July!AH14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>485</v>
+        <v>526</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3068,11 +3068,11 @@
       </c>
       <c r="G29" s="5">
         <f t="shared" si="1"/>
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H29" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="I29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>485</v>
+        <v>526</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -12684,10 +12684,12 @@
         <v>4</v>
       </c>
       <c r="AF14" s="18"/>
-      <c r="AG14" s="54"/>
+      <c r="AG14" s="54">
+        <v>3</v>
+      </c>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -13797,17 +13799,37 @@
         <f>January!B14</f>
         <v>AI-Driven Agentic Orchestration Software (AOC-WebAPI)</v>
       </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
+      <c r="C14" s="41">
+        <v>4</v>
+      </c>
+      <c r="D14" s="17">
+        <v>3</v>
+      </c>
+      <c r="E14" s="17">
+        <v>2</v>
+      </c>
       <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
-      <c r="M14" s="17"/>
+      <c r="G14" s="17">
+        <v>5</v>
+      </c>
+      <c r="H14" s="18">
+        <v>2</v>
+      </c>
+      <c r="I14" s="16">
+        <v>4</v>
+      </c>
+      <c r="J14" s="17">
+        <v>4</v>
+      </c>
+      <c r="K14" s="17">
+        <v>4</v>
+      </c>
+      <c r="L14" s="17">
+        <v>4</v>
+      </c>
+      <c r="M14" s="17">
+        <v>6</v>
+      </c>
       <c r="N14" s="17"/>
       <c r="O14" s="18"/>
       <c r="P14" s="16"/>
@@ -13829,7 +13851,7 @@
       <c r="AF14" s="20"/>
       <c r="AG14" s="43">
         <f t="shared" ref="AG14:AG30" si="0">SUM(C14:AF14)</f>
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:33" ht="15" customHeight="1">
@@ -16975,17 +16997,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17220,6 +17231,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -17230,19 +17252,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17261,6 +17270,19 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Add JWT capability enforcement
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{521992A5-7392-C54B-912C-07EBCFC6EF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DE459C-90BE-6C4C-8A9E-86E4E0C9C45B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27720" yWindow="-20820" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="H12" s="70">
         <f>June!AG14</f>
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="I12" s="70">
         <f>July!AH14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>526</v>
+        <v>572</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="H29" s="5">
         <f t="shared" si="1"/>
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="I29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>526</v>
+        <v>572</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -13831,16 +13831,36 @@
         <v>6</v>
       </c>
       <c r="N14" s="17"/>
-      <c r="O14" s="18"/>
-      <c r="P14" s="16"/>
-      <c r="Q14" s="17"/>
-      <c r="R14" s="17"/>
-      <c r="S14" s="17"/>
-      <c r="T14" s="17"/>
-      <c r="U14" s="17"/>
-      <c r="V14" s="18"/>
-      <c r="W14" s="16"/>
-      <c r="X14" s="17"/>
+      <c r="O14" s="18">
+        <v>4</v>
+      </c>
+      <c r="P14" s="16">
+        <v>6</v>
+      </c>
+      <c r="Q14" s="17">
+        <v>5</v>
+      </c>
+      <c r="R14" s="17">
+        <v>5</v>
+      </c>
+      <c r="S14" s="17">
+        <v>6</v>
+      </c>
+      <c r="T14" s="17">
+        <v>6</v>
+      </c>
+      <c r="U14" s="17">
+        <v>4</v>
+      </c>
+      <c r="V14" s="18">
+        <v>3</v>
+      </c>
+      <c r="W14" s="16">
+        <v>3</v>
+      </c>
+      <c r="X14" s="17">
+        <v>4</v>
+      </c>
       <c r="Y14" s="17"/>
       <c r="Z14" s="17"/>
       <c r="AA14" s="17"/>
@@ -13851,7 +13871,7 @@
       <c r="AF14" s="20"/>
       <c r="AG14" s="43">
         <f t="shared" ref="AG14:AG30" si="0">SUM(C14:AF14)</f>
-        <v>38</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:33" ht="15" customHeight="1">
@@ -16997,6 +17017,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17231,17 +17262,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -17252,6 +17272,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17270,19 +17303,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Add pooled sandbox executor and benchmark CLI
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10621"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DE459C-90BE-6C4C-8A9E-86E4E0C9C45B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{584C010D-BE54-1446-B180-9BCE5A530B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27720" yWindow="-20820" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="19340" tabRatio="666" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -1368,15 +1368,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1391,6 +1382,15 @@
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1931,53 +1931,53 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:34" ht="58.5" customHeight="1">
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="94"/>
-      <c r="M2" s="94"/>
-      <c r="N2" s="94"/>
-      <c r="O2" s="94"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="91"/>
+      <c r="K2" s="91"/>
+      <c r="L2" s="91"/>
+      <c r="M2" s="91"/>
+      <c r="N2" s="91"/>
+      <c r="O2" s="91"/>
       <c r="R2" s="36"/>
       <c r="U2" s="36"/>
       <c r="X2" s="36"/>
     </row>
     <row r="3" spans="1:34" ht="24.75" customHeight="1">
-      <c r="A3" s="93" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="93"/>
-      <c r="C3" s="93"/>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93"/>
+      <c r="A3" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
+      <c r="M3" s="90"/>
+      <c r="N3" s="90"/>
+      <c r="O3" s="90"/>
     </row>
     <row r="4" spans="1:34" ht="15" customHeight="1">
-      <c r="A4" s="93"/>
-      <c r="B4" s="93"/>
-      <c r="C4" s="93"/>
-      <c r="D4" s="93"/>
-      <c r="E4" s="93"/>
-      <c r="F4" s="93"/>
-      <c r="G4" s="93"/>
-      <c r="H4" s="93"/>
-      <c r="I4" s="93"/>
-      <c r="J4" s="93"/>
-      <c r="K4" s="93"/>
-      <c r="L4" s="93"/>
-      <c r="M4" s="93"/>
-      <c r="N4" s="93"/>
-      <c r="O4" s="93"/>
+      <c r="A4" s="90"/>
+      <c r="B4" s="90"/>
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="90"/>
+      <c r="L4" s="90"/>
+      <c r="M4" s="90"/>
+      <c r="N4" s="90"/>
+      <c r="O4" s="90"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="B6" s="77" t="s">
@@ -1989,15 +1989,15 @@
       <c r="B7" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="90" t="s">
+      <c r="E7" s="87" t="s">
         <v>48</v>
       </c>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="91"/>
-      <c r="K7" s="92"/>
+      <c r="F7" s="88"/>
+      <c r="G7" s="88"/>
+      <c r="H7" s="88"/>
+      <c r="I7" s="88"/>
+      <c r="J7" s="88"/>
+      <c r="K7" s="89"/>
       <c r="L7" s="79"/>
       <c r="AH7" s="2"/>
     </row>
@@ -2005,15 +2005,15 @@
       <c r="B8" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="90" t="s">
+      <c r="E8" s="87" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="91"/>
-      <c r="G8" s="91"/>
-      <c r="H8" s="91"/>
-      <c r="I8" s="91"/>
-      <c r="J8" s="91"/>
-      <c r="K8" s="92"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="88"/>
+      <c r="K8" s="89"/>
       <c r="L8" s="79"/>
       <c r="AH8" s="2"/>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="H12" s="70">
         <f>June!AG14</f>
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="I12" s="70">
         <f>July!AH14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>572</v>
+        <v>596</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="H29" s="5">
         <f t="shared" si="1"/>
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="I29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>572</v>
+        <v>596</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -3198,34 +3198,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -3236,32 +3236,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -4326,34 +4326,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -4364,32 +4364,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -5473,34 +5473,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -5511,32 +5511,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -6596,34 +6596,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -6634,32 +6634,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -7750,34 +7750,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:37" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:37" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -7788,32 +7788,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:37" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:37" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -8911,34 +8911,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:31" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:31" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -8949,32 +8949,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:31" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:31" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -10031,34 +10031,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -10069,32 +10069,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -11229,34 +11229,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -11267,32 +11267,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -12396,34 +12396,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -12434,32 +12434,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87" t="s">
+      <c r="C9" s="92" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -13595,34 +13595,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -13633,32 +13633,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -13861,17 +13861,31 @@
       <c r="X14" s="17">
         <v>4</v>
       </c>
-      <c r="Y14" s="17"/>
-      <c r="Z14" s="17"/>
-      <c r="AA14" s="17"/>
-      <c r="AB14" s="17"/>
-      <c r="AC14" s="18"/>
-      <c r="AD14" s="16"/>
-      <c r="AE14" s="17"/>
+      <c r="Y14" s="17">
+        <v>2</v>
+      </c>
+      <c r="Z14" s="17">
+        <v>2</v>
+      </c>
+      <c r="AA14" s="17">
+        <v>4</v>
+      </c>
+      <c r="AB14" s="17">
+        <v>4</v>
+      </c>
+      <c r="AC14" s="18">
+        <v>4</v>
+      </c>
+      <c r="AD14" s="16">
+        <v>2</v>
+      </c>
+      <c r="AE14" s="17">
+        <v>6</v>
+      </c>
       <c r="AF14" s="20"/>
       <c r="AG14" s="43">
         <f t="shared" ref="AG14:AG30" si="0">SUM(C14:AF14)</f>
-        <v>84</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:33" ht="15" customHeight="1">
@@ -14757,34 +14771,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -14795,32 +14809,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -15907,34 +15921,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="92" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="87" t="str">
+      <c r="C6" s="92" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="89"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -15945,32 +15959,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="92" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="94"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="87">
+      <c r="C9" s="92">
         <v>2026</v>
       </c>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="89"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="94"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>

</xml_diff>

<commit_message>
Add process-backed sandbox slot, replacing in-process stub with real subprocess isolation for July hardening.
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10703"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{584C010D-BE54-1446-B180-9BCE5A530B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{776F3041-1B87-F245-9B7D-90872165A0F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="19340" tabRatio="666" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -1368,6 +1368,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1382,15 +1391,6 @@
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1931,53 +1931,53 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:34" ht="58.5" customHeight="1">
-      <c r="H2" s="91"/>
-      <c r="I2" s="91"/>
-      <c r="J2" s="91"/>
-      <c r="K2" s="91"/>
-      <c r="L2" s="91"/>
-      <c r="M2" s="91"/>
-      <c r="N2" s="91"/>
-      <c r="O2" s="91"/>
+      <c r="H2" s="94"/>
+      <c r="I2" s="94"/>
+      <c r="J2" s="94"/>
+      <c r="K2" s="94"/>
+      <c r="L2" s="94"/>
+      <c r="M2" s="94"/>
+      <c r="N2" s="94"/>
+      <c r="O2" s="94"/>
       <c r="R2" s="36"/>
       <c r="U2" s="36"/>
       <c r="X2" s="36"/>
     </row>
     <row r="3" spans="1:34" ht="24.75" customHeight="1">
-      <c r="A3" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="90"/>
-      <c r="K3" s="90"/>
-      <c r="L3" s="90"/>
-      <c r="M3" s="90"/>
-      <c r="N3" s="90"/>
-      <c r="O3" s="90"/>
+      <c r="A3" s="93" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="93"/>
+      <c r="C3" s="93"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="93"/>
+      <c r="J3" s="93"/>
+      <c r="K3" s="93"/>
+      <c r="L3" s="93"/>
+      <c r="M3" s="93"/>
+      <c r="N3" s="93"/>
+      <c r="O3" s="93"/>
     </row>
     <row r="4" spans="1:34" ht="15" customHeight="1">
-      <c r="A4" s="90"/>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="90"/>
-      <c r="I4" s="90"/>
-      <c r="J4" s="90"/>
-      <c r="K4" s="90"/>
-      <c r="L4" s="90"/>
-      <c r="M4" s="90"/>
-      <c r="N4" s="90"/>
-      <c r="O4" s="90"/>
+      <c r="A4" s="93"/>
+      <c r="B4" s="93"/>
+      <c r="C4" s="93"/>
+      <c r="D4" s="93"/>
+      <c r="E4" s="93"/>
+      <c r="F4" s="93"/>
+      <c r="G4" s="93"/>
+      <c r="H4" s="93"/>
+      <c r="I4" s="93"/>
+      <c r="J4" s="93"/>
+      <c r="K4" s="93"/>
+      <c r="L4" s="93"/>
+      <c r="M4" s="93"/>
+      <c r="N4" s="93"/>
+      <c r="O4" s="93"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="B6" s="77" t="s">
@@ -1989,15 +1989,15 @@
       <c r="B7" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="87" t="s">
+      <c r="E7" s="90" t="s">
         <v>48</v>
       </c>
-      <c r="F7" s="88"/>
-      <c r="G7" s="88"/>
-      <c r="H7" s="88"/>
-      <c r="I7" s="88"/>
-      <c r="J7" s="88"/>
-      <c r="K7" s="89"/>
+      <c r="F7" s="91"/>
+      <c r="G7" s="91"/>
+      <c r="H7" s="91"/>
+      <c r="I7" s="91"/>
+      <c r="J7" s="91"/>
+      <c r="K7" s="92"/>
       <c r="L7" s="79"/>
       <c r="AH7" s="2"/>
     </row>
@@ -2005,15 +2005,15 @@
       <c r="B8" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="87" t="s">
+      <c r="E8" s="90" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="88"/>
-      <c r="K8" s="89"/>
+      <c r="F8" s="91"/>
+      <c r="G8" s="91"/>
+      <c r="H8" s="91"/>
+      <c r="I8" s="91"/>
+      <c r="J8" s="91"/>
+      <c r="K8" s="92"/>
       <c r="L8" s="79"/>
       <c r="AH8" s="2"/>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="I12" s="70">
         <f>July!AH14</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J12" s="70">
         <f>August!AH14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>596</v>
+        <v>631</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="I29" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>596</v>
+        <v>631</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -3198,34 +3198,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -3236,32 +3236,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -4326,34 +4326,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -4364,32 +4364,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -5473,34 +5473,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -5511,32 +5511,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -6596,34 +6596,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -6634,32 +6634,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -7750,34 +7750,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:37" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:37" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -7788,32 +7788,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:37" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:37" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -8911,34 +8911,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:31" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:31" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -8949,32 +8949,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:31" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:31" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -10031,34 +10031,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -10069,32 +10069,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -11229,34 +11229,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -11267,32 +11267,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -12396,34 +12396,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -12434,32 +12434,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92" t="s">
+      <c r="C9" s="87" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -13595,34 +13595,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:33" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -13633,32 +13633,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:33" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -14771,34 +14771,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -14809,32 +14809,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -14982,14 +14982,28 @@
         <f>January!B14</f>
         <v>AI-Driven Agentic Orchestration Software (AOC-WebAPI)</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
+      <c r="C14" s="17">
+        <v>6</v>
+      </c>
+      <c r="D14" s="17">
+        <v>6</v>
+      </c>
+      <c r="E14" s="17">
+        <v>4</v>
+      </c>
       <c r="F14" s="18"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
+      <c r="G14" s="16">
+        <v>2</v>
+      </c>
+      <c r="H14" s="17">
+        <v>6</v>
+      </c>
+      <c r="I14" s="17">
+        <v>5</v>
+      </c>
+      <c r="J14" s="17">
+        <v>6</v>
+      </c>
       <c r="K14" s="17"/>
       <c r="L14" s="17"/>
       <c r="M14" s="18"/>
@@ -15015,7 +15029,7 @@
       <c r="AG14" s="20"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -15921,34 +15935,34 @@
         <v>2</v>
       </c>
       <c r="B5" s="78"/>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="87" t="str">
         <f>Overview!E7</f>
         <v>Filippo Margiotta | 265126642</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="94"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:34" ht="15" customHeight="1">
       <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="C6" s="92" t="str">
+      <c r="C6" s="87" t="str">
         <f>Overview!E8</f>
         <v>Director / Architect</v>
       </c>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
+      <c r="H6" s="88"/>
+      <c r="I6" s="88"/>
+      <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:34" ht="15" customHeight="1">
       <c r="A7" s="78"/>
@@ -15959,32 +15973,32 @@
         <v>19</v>
       </c>
       <c r="B8" s="78"/>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="87" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="94"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
     </row>
     <row r="9" spans="1:34" ht="15" customHeight="1">
       <c r="A9" s="77" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="C9" s="92">
+      <c r="C9" s="87">
         <v>2026</v>
       </c>
-      <c r="D9" s="93"/>
-      <c r="E9" s="93"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="94"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="88"/>
+      <c r="F9" s="88"/>
+      <c r="G9" s="88"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="89"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1">
       <c r="A11" s="3"/>
@@ -17042,6 +17056,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17276,15 +17299,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
   <ds:schemaRefs>
@@ -17299,6 +17313,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17317,14 +17339,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Sandbox hardening with container isolation and deterministic failure replay
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10726"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{776F3041-1B87-F245-9B7D-90872165A0F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C3AF47F-D7B2-4842-9B9A-85C3363915DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2091,11 +2091,11 @@
       </c>
       <c r="I12" s="70">
         <f>July!AH14</f>
-        <v>35</v>
+        <v>79</v>
       </c>
       <c r="J12" s="70">
         <f>August!AH14</f>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="K12" s="70">
         <f>September!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>631</v>
+        <v>689</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3076,11 +3076,11 @@
       </c>
       <c r="I29" s="5">
         <f t="shared" si="1"/>
-        <v>35</v>
+        <v>79</v>
       </c>
       <c r="J29" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="K29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>631</v>
+        <v>689</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -15004,22 +15004,46 @@
       <c r="J14" s="17">
         <v>6</v>
       </c>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
-      <c r="M14" s="18"/>
-      <c r="N14" s="16"/>
-      <c r="O14" s="17"/>
-      <c r="P14" s="17"/>
-      <c r="Q14" s="17"/>
-      <c r="R14" s="17"/>
+      <c r="K14" s="17">
+        <v>6</v>
+      </c>
+      <c r="L14" s="17">
+        <v>4</v>
+      </c>
+      <c r="M14" s="18">
+        <v>2</v>
+      </c>
+      <c r="N14" s="16">
+        <v>2</v>
+      </c>
+      <c r="O14" s="17">
+        <v>4</v>
+      </c>
+      <c r="P14" s="17">
+        <v>6</v>
+      </c>
+      <c r="Q14" s="17">
+        <v>3</v>
+      </c>
+      <c r="R14" s="17">
+        <v>1</v>
+      </c>
       <c r="S14" s="17"/>
       <c r="T14" s="18"/>
       <c r="U14" s="16"/>
-      <c r="V14" s="17"/>
-      <c r="W14" s="17"/>
+      <c r="V14" s="17">
+        <v>6</v>
+      </c>
+      <c r="W14" s="17">
+        <v>4</v>
+      </c>
       <c r="X14" s="17"/>
-      <c r="Y14" s="17"/>
-      <c r="Z14" s="17"/>
+      <c r="Y14" s="17">
+        <v>2</v>
+      </c>
+      <c r="Z14" s="17">
+        <v>4</v>
+      </c>
       <c r="AA14" s="18"/>
       <c r="AB14" s="16"/>
       <c r="AC14" s="17"/>
@@ -15029,7 +15053,7 @@
       <c r="AG14" s="20"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>35</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -16142,9 +16166,15 @@
         <v>AI-Driven Agentic Orchestration Software (AOC-WebAPI)</v>
       </c>
       <c r="C14" s="58"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
+      <c r="D14" s="16">
+        <v>6</v>
+      </c>
+      <c r="E14" s="17">
+        <v>6</v>
+      </c>
+      <c r="F14" s="17">
+        <v>2</v>
+      </c>
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
@@ -16174,7 +16204,7 @@
       <c r="AG14" s="20"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -17056,15 +17086,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17299,6 +17320,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
   <ds:schemaRefs>
@@ -17313,14 +17343,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17339,6 +17361,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Add deterministic planner contracts, validation, and playbook retrieval
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10802"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C3AF47F-D7B2-4842-9B9A-85C3363915DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8F55E7-0F3F-2A43-9EAF-CE58F909C169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="33320" windowHeight="17620" tabRatio="666" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="J12" s="70">
         <f>August!AH14</f>
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="K12" s="70">
         <f>September!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>689</v>
+        <v>721</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3080,7 +3080,7 @@
       </c>
       <c r="J29" s="5">
         <f t="shared" si="1"/>
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="K29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>689</v>
+        <v>721</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -16176,16 +16176,32 @@
         <v>2</v>
       </c>
       <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
+      <c r="H14" s="17">
+        <v>6</v>
+      </c>
+      <c r="I14" s="17">
+        <v>2</v>
+      </c>
       <c r="J14" s="18"/>
-      <c r="K14" s="16"/>
+      <c r="K14" s="16">
+        <v>4</v>
+      </c>
       <c r="L14" s="17"/>
-      <c r="M14" s="17"/>
-      <c r="N14" s="17"/>
-      <c r="O14" s="17"/>
-      <c r="P14" s="17"/>
-      <c r="Q14" s="18"/>
+      <c r="M14" s="17">
+        <v>4</v>
+      </c>
+      <c r="N14" s="17">
+        <v>4</v>
+      </c>
+      <c r="O14" s="17">
+        <v>4</v>
+      </c>
+      <c r="P14" s="17">
+        <v>6</v>
+      </c>
+      <c r="Q14" s="18">
+        <v>2</v>
+      </c>
       <c r="R14" s="16"/>
       <c r="S14" s="17"/>
       <c r="T14" s="17"/>
@@ -16204,7 +16220,7 @@
       <c r="AG14" s="20"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>14</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -17086,6 +17102,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17320,15 +17345,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
   <ds:schemaRefs>
@@ -17343,6 +17359,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17361,14 +17385,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Add deterministic planner orchestration, capability-protected step execution, and signed replay
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10810"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8F55E7-0F3F-2A43-9EAF-CE58F909C169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE9F975-D970-DC42-98A0-07B9327A252A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="33320" windowHeight="17620" tabRatio="666" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="J12" s="70">
         <f>August!AH14</f>
-        <v>46</v>
+        <v>97</v>
       </c>
       <c r="K12" s="70">
         <f>September!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>721</v>
+        <v>772</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3080,7 +3080,7 @@
       </c>
       <c r="J29" s="5">
         <f t="shared" si="1"/>
-        <v>46</v>
+        <v>97</v>
       </c>
       <c r="K29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>721</v>
+        <v>772</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -16203,24 +16203,48 @@
         <v>2</v>
       </c>
       <c r="R14" s="16"/>
-      <c r="S14" s="17"/>
-      <c r="T14" s="17"/>
-      <c r="U14" s="17"/>
-      <c r="V14" s="17"/>
-      <c r="W14" s="17"/>
-      <c r="X14" s="18"/>
-      <c r="Y14" s="16"/>
+      <c r="S14" s="17">
+        <v>4</v>
+      </c>
+      <c r="T14" s="17">
+        <v>6</v>
+      </c>
+      <c r="U14" s="17">
+        <v>3</v>
+      </c>
+      <c r="V14" s="17">
+        <v>5</v>
+      </c>
+      <c r="W14" s="17">
+        <v>4</v>
+      </c>
+      <c r="X14" s="18">
+        <v>2</v>
+      </c>
+      <c r="Y14" s="16">
+        <v>3</v>
+      </c>
       <c r="Z14" s="17"/>
-      <c r="AA14" s="17"/>
+      <c r="AA14" s="17">
+        <v>5</v>
+      </c>
       <c r="AB14" s="17"/>
-      <c r="AC14" s="17"/>
-      <c r="AD14" s="17"/>
+      <c r="AC14" s="17">
+        <v>6</v>
+      </c>
+      <c r="AD14" s="17">
+        <v>3</v>
+      </c>
       <c r="AE14" s="18"/>
-      <c r="AF14" s="16"/>
-      <c r="AG14" s="20"/>
+      <c r="AF14" s="16">
+        <v>4</v>
+      </c>
+      <c r="AG14" s="20">
+        <v>6</v>
+      </c>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>46</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -17091,26 +17115,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17345,28 +17349,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17385,6 +17388,27 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>